<commit_message>
update for input ircs control 2
</commit_message>
<xml_diff>
--- a/IRCS2_build/Input Sheet.xlsx
+++ b/IRCS2_build/Input Sheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GITHUB\IRCS\IRCS2_build\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\13. Employee Folder\Christo\control 2\11M\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{417A8471-B222-4E81-9A27-E1D6B3E1A263}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0D9EEA4-8496-46B8-A61E-FC12976430D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{1CB29936-90A1-4B24-80D1-9DB6A66D7875}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="8" xr2:uid="{1CB29936-90A1-4B24-80D1-9DB6A66D7875}"/>
   </bookViews>
   <sheets>
     <sheet name="PATH INPUT" sheetId="7" r:id="rId1"/>
@@ -20,8 +20,9 @@
     <sheet name="SPEC UL" sheetId="6" r:id="rId5"/>
     <sheet name="TRAD" sheetId="8" r:id="rId6"/>
     <sheet name="SPEC TRAD" sheetId="9" r:id="rId7"/>
-    <sheet name="Campaign Lookup" sheetId="10" r:id="rId8"/>
-    <sheet name="Code BSI" sheetId="11" r:id="rId9"/>
+    <sheet name="AZCP" sheetId="12" r:id="rId8"/>
+    <sheet name="LGC LGM Campaign Lookup" sheetId="13" r:id="rId9"/>
+    <sheet name="Code BSI" sheetId="11" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">UL!$A$1:$B$151</definedName>
@@ -47,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="588" uniqueCount="505">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="602" uniqueCount="514">
   <si>
     <t>Prophet Code</t>
   </si>
@@ -1522,56 +1523,84 @@
     <t>4_IDR</t>
   </si>
   <si>
-    <t>P:\13. Employee Folder\Christo\8M\DV_AZTRAD_Stat.csv</t>
-  </si>
-  <si>
-    <t>P:\13. Employee Folder\Christo\8M\DV_AZUL_Stat_8M25.csv</t>
-  </si>
-  <si>
-    <t>P:\13. Employee Folder\Christo\8M\IT_AZTRAD_FULL_Stat.csv</t>
-  </si>
-  <si>
-    <t>P:\13. Employee Folder\Christo\8M\IT_AZUL_FULL_Stat_8M25.csv</t>
-  </si>
-  <si>
-    <t>P:\13. Employee Folder\Christo\8M\Summary.csv</t>
-  </si>
-  <si>
-    <t>P:\13. Employee Folder\Christo\8M\LGC_LGM_Campaign_Aug25.txt</t>
-  </si>
-  <si>
-    <t>P:\13. Employee Folder\Christo\8M\BSI_ATTRIBUSI_020925.xlsx</t>
-  </si>
-  <si>
-    <t>P:\13. Employee Folder\Christo\8M\RESERVE_TRADCONV_RWNB_IFRS_20250902.txt</t>
-  </si>
-  <si>
-    <t>P:\13. Employee Folder\Christo\8M\RESERVE_TRADSHA_RWNB_IFRS_20250902.txt</t>
-  </si>
-  <si>
     <t>ULMGRW</t>
   </si>
   <si>
     <t>MYGRW</t>
   </si>
   <si>
-    <t>Control IFRS 17.2_8M2025_UAT</t>
-  </si>
-  <si>
     <t>ACP Campaign</t>
   </si>
   <si>
-    <t>P:\13. Employee Folder\Christo\8M\ACP_campaign_Aug25.txt</t>
+    <t>HPRHA</t>
+  </si>
+  <si>
+    <t>CPRHA_</t>
+  </si>
+  <si>
+    <t>CWFTIN</t>
+  </si>
+  <si>
+    <t>AZFI</t>
+  </si>
+  <si>
+    <t>P:\13. Employee Folder\Christo\control 2\11M\DV_AZTRAD_Stat.csv</t>
+  </si>
+  <si>
+    <t>P:\13. Employee Folder\Christo\control 2\11M\DV_AZUL_Stat_11M.csv</t>
+  </si>
+  <si>
+    <t>P:\13. Employee Folder\Christo\control 2\11M\IT_AZTRAD_FULL_Stat.csv</t>
+  </si>
+  <si>
+    <t>P:\13. Employee Folder\Christo\control 2\11M\IT_AZUL_FULL_Stat.csv</t>
+  </si>
+  <si>
+    <t>P:\13. Employee Folder\Christo\control 2\11M\Summary.csv</t>
+  </si>
+  <si>
+    <t>P:\13. Employee Folder\Christo\control 2\11M\LGC_LGM_Camp_Nov25.txt</t>
+  </si>
+  <si>
+    <t>P:\13. Employee Folder\Christo\control 2\11M\BSI_ATTRIBUSI_021225.xlsx</t>
+  </si>
+  <si>
+    <t>P:\13. Employee Folder\Christo\control 2\11M\ACP_Camp_Nov25.txt</t>
+  </si>
+  <si>
+    <t>P:\13. Employee Folder\Christo\control 2\11M\RESERVE_TRADCONV_RWNB_IFRS_20251202.txt</t>
+  </si>
+  <si>
+    <t>P:\13. Employee Folder\Christo\control 2\11M\RESERVE_TRADSHA_RWNB_IFRS_20251202.txt</t>
+  </si>
+  <si>
+    <t>Bonus</t>
+  </si>
+  <si>
+    <t>Batch</t>
+  </si>
+  <si>
+    <t>Control IFRS 17.2_11M2025_test</t>
+  </si>
+  <si>
+    <t>Greater than Or Equal To</t>
+  </si>
+  <si>
+    <t>0.1</t>
+  </si>
+  <si>
+    <t>%SA bonus</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\)_);_(* &quot;-&quot;_);_(@_)"/>
   </numFmts>
-  <fonts count="23" x14ac:knownFonts="1">
+  <fonts count="24" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1737,6 +1766,14 @@
     <font>
       <b/>
       <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -2066,7 +2103,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="42">
+  <cellStyleXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
@@ -2109,8 +2146,9 @@
     <xf numFmtId="0" fontId="3" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2118,19 +2156,40 @@
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="3" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="22" fillId="34" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="18" fillId="34" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="34" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="34" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="42" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="42" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="42" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="42">
+  <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
     <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
     <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
@@ -2158,6 +2217,7 @@
     <cellStyle name="Bad" xfId="7" builtinId="27" customBuiltin="1"/>
     <cellStyle name="Calculation" xfId="11" builtinId="22" customBuiltin="1"/>
     <cellStyle name="Check Cell" xfId="13" builtinId="23" customBuiltin="1"/>
+    <cellStyle name="Comma" xfId="42" builtinId="3"/>
     <cellStyle name="Explanatory Text" xfId="16" builtinId="53" customBuiltin="1"/>
     <cellStyle name="Good" xfId="6" builtinId="26" customBuiltin="1"/>
     <cellStyle name="Heading 1" xfId="2" builtinId="16" customBuiltin="1"/>
@@ -2504,7 +2564,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA018573-BF85-417A-8309-CECE2ACCAF79}">
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="34.21875" bestFit="1" customWidth="1"/>
@@ -2524,7 +2584,7 @@
         <v>485</v>
       </c>
       <c r="B2" s="4">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -2540,7 +2600,7 @@
         <v>450</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>491</v>
+        <v>498</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
@@ -2548,7 +2608,7 @@
         <v>451</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>492</v>
+        <v>499</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
@@ -2556,7 +2616,7 @@
         <v>453</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>493</v>
+        <v>500</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
@@ -2564,7 +2624,7 @@
         <v>452</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>494</v>
+        <v>501</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
@@ -2572,7 +2632,7 @@
         <v>479</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>495</v>
+        <v>502</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
@@ -2580,7 +2640,7 @@
         <v>480</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>496</v>
+        <v>503</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
@@ -2588,15 +2648,15 @@
         <v>481</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>497</v>
+        <v>504</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>503</v>
+        <v>493</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
@@ -2604,7 +2664,7 @@
         <v>483</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>498</v>
+        <v>506</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
@@ -2612,7 +2672,7 @@
         <v>484</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>499</v>
+        <v>507</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
@@ -2620,11 +2680,42 @@
         <v>454</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>502</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B15" s="15"/>
+        <v>510</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32AEBD3E-E17A-4FD7-BDAF-3A1BA4999487}">
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>475</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>477</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>478</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>426</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2679,1219 +2770,1219 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="10" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="9" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="9" t="s">
         <v>252</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="9" t="s">
         <v>253</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="9" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="B5" s="12" t="s">
+      <c r="B5" s="9" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A6" s="12" t="s">
+      <c r="A6" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="B6" s="12" t="s">
+      <c r="B6" s="9" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A7" s="12" t="s">
+      <c r="A7" s="9" t="s">
         <v>222</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="B7" s="9" t="s">
         <v>223</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A8" s="12" t="s">
+      <c r="A8" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="12" t="s">
+      <c r="B8" s="9" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="B9" s="9" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A10" s="12" t="s">
+      <c r="A10" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="12" t="s">
+      <c r="B10" s="9" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A11" s="12" t="s">
+      <c r="A11" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="B11" s="12" t="s">
+      <c r="B11" s="9" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A12" s="12" t="s">
+      <c r="A12" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="12" t="s">
+      <c r="B12" s="9" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A13" s="12" t="s">
+      <c r="A13" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="B13" s="12" t="s">
+      <c r="B13" s="9" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A14" s="12" t="s">
+      <c r="A14" s="9" t="s">
         <v>431</v>
       </c>
-      <c r="B14" s="12" t="s">
+      <c r="B14" s="9" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A15" s="12" t="s">
+      <c r="A15" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="12" t="s">
+      <c r="B15" s="9" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A16" s="12" t="s">
+      <c r="A16" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="12" t="s">
+      <c r="B16" s="9" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A17" s="12" t="s">
+      <c r="A17" s="9" t="s">
         <v>230</v>
       </c>
-      <c r="B17" s="12" t="s">
+      <c r="B17" s="9" t="s">
         <v>231</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="12" t="s">
+      <c r="A18" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="B18" s="12" t="s">
+      <c r="B18" s="9" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A19" s="12" t="s">
+      <c r="A19" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="B19" s="12" t="s">
+      <c r="B19" s="9" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A20" s="12" t="s">
+      <c r="A20" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="B20" s="12" t="s">
+      <c r="B20" s="9" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A21" s="12" t="s">
+      <c r="A21" s="9" t="s">
         <v>432</v>
       </c>
-      <c r="B21" s="12" t="s">
+      <c r="B21" s="9" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A22" s="12" t="s">
+      <c r="A22" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="B22" s="12" t="s">
+      <c r="B22" s="9" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A23" s="12" t="s">
+      <c r="A23" s="9" t="s">
         <v>433</v>
       </c>
-      <c r="B23" s="12" t="s">
+      <c r="B23" s="9" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A24" s="12" t="s">
+      <c r="A24" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="B24" s="12" t="s">
+      <c r="B24" s="9" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A25" s="12" t="s">
+      <c r="A25" s="9" t="s">
         <v>198</v>
       </c>
-      <c r="B25" s="12" t="s">
+      <c r="B25" s="9" t="s">
         <v>199</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A26" s="12" t="s">
+      <c r="A26" s="9" t="s">
         <v>200</v>
       </c>
-      <c r="B26" s="12" t="s">
+      <c r="B26" s="9" t="s">
         <v>201</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A27" s="12" t="s">
+      <c r="A27" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="B27" s="12" t="s">
+      <c r="B27" s="9" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A28" s="12" t="s">
+      <c r="A28" s="9" t="s">
         <v>434</v>
       </c>
-      <c r="B28" s="12" t="s">
+      <c r="B28" s="9" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A29" s="12" t="s">
+      <c r="A29" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="B29" s="12" t="s">
+      <c r="B29" s="9" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A30" s="12" t="s">
+      <c r="A30" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="B30" s="12" t="s">
+      <c r="B30" s="9" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A31" s="12" t="s">
+      <c r="A31" s="9" t="s">
         <v>248</v>
       </c>
-      <c r="B31" s="12" t="s">
+      <c r="B31" s="9" t="s">
         <v>249</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A32" s="12" t="s">
+      <c r="A32" s="9" t="s">
         <v>250</v>
       </c>
-      <c r="B32" s="12" t="s">
+      <c r="B32" s="9" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A33" s="12" t="s">
+      <c r="A33" s="9" t="s">
         <v>258</v>
       </c>
-      <c r="B33" s="12" t="s">
+      <c r="B33" s="9" t="s">
         <v>259</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A34" s="12" t="s">
+      <c r="A34" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="B34" s="12" t="s">
+      <c r="B34" s="9" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A35" s="12" t="s">
+      <c r="A35" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="B35" s="12" t="s">
+      <c r="B35" s="9" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A36" s="12" t="s">
+      <c r="A36" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="B36" s="12" t="s">
+      <c r="B36" s="9" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A37" s="12" t="s">
+      <c r="A37" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="B37" s="12" t="s">
+      <c r="B37" s="9" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A38" s="12" t="s">
+      <c r="A38" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="B38" s="12" t="s">
+      <c r="B38" s="9" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A39" s="12" t="s">
+      <c r="A39" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="B39" s="12" t="s">
+      <c r="B39" s="9" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A40" s="12" t="s">
+      <c r="A40" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="B40" s="12" t="s">
+      <c r="B40" s="9" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A41" s="12" t="s">
+      <c r="A41" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="B41" s="12" t="s">
+      <c r="B41" s="9" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A42" s="12" t="s">
+      <c r="A42" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="B42" s="12" t="s">
+      <c r="B42" s="9" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A43" s="12" t="s">
+      <c r="A43" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="B43" s="12" t="s">
+      <c r="B43" s="9" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A44" s="12" t="s">
+      <c r="A44" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="B44" s="12" t="s">
+      <c r="B44" s="9" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A45" s="12" t="s">
+      <c r="A45" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="B45" s="12" t="s">
+      <c r="B45" s="9" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A46" s="12" t="s">
+      <c r="A46" s="9" t="s">
         <v>224</v>
       </c>
-      <c r="B46" s="12" t="s">
+      <c r="B46" s="9" t="s">
         <v>225</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A47" s="12" t="s">
+      <c r="A47" s="9" t="s">
         <v>256</v>
       </c>
-      <c r="B47" s="12" t="s">
+      <c r="B47" s="9" t="s">
         <v>257</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A48" s="12" t="s">
+      <c r="A48" s="9" t="s">
         <v>232</v>
       </c>
-      <c r="B48" s="12" t="s">
+      <c r="B48" s="9" t="s">
         <v>233</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A49" s="12" t="s">
+      <c r="A49" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="B49" s="12" t="s">
+      <c r="B49" s="9" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A50" s="12" t="s">
+      <c r="A50" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="B50" s="12" t="s">
+      <c r="B50" s="9" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A51" s="12" t="s">
+      <c r="A51" s="9" t="s">
         <v>234</v>
       </c>
-      <c r="B51" s="12" t="s">
+      <c r="B51" s="9" t="s">
         <v>235</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A52" s="12" t="s">
+      <c r="A52" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="B52" s="12" t="s">
+      <c r="B52" s="9" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A53" s="12" t="s">
+      <c r="A53" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="B53" s="12" t="s">
+      <c r="B53" s="9" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A54" s="12" t="s">
+      <c r="A54" s="9" t="s">
         <v>236</v>
       </c>
-      <c r="B54" s="12" t="s">
+      <c r="B54" s="9" t="s">
         <v>237</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A55" s="12" t="s">
+      <c r="A55" s="9" t="s">
         <v>265</v>
       </c>
-      <c r="B55" s="12" t="s">
+      <c r="B55" s="9" t="s">
         <v>266</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A56" s="12" t="s">
+      <c r="A56" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="B56" s="12" t="s">
+      <c r="B56" s="9" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A57" s="12" t="s">
+      <c r="A57" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="B57" s="12" t="s">
+      <c r="B57" s="9" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A58" s="12" t="s">
+      <c r="A58" s="9" t="s">
         <v>238</v>
       </c>
-      <c r="B58" s="12" t="s">
+      <c r="B58" s="9" t="s">
         <v>239</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A59" s="12" t="s">
+      <c r="A59" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="B59" s="12" t="s">
+      <c r="B59" s="9" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A60" s="12" t="s">
+      <c r="A60" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="B60" s="12" t="s">
+      <c r="B60" s="9" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A61" s="12" t="s">
+      <c r="A61" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="B61" s="12" t="s">
+      <c r="B61" s="9" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A62" s="12" t="s">
+      <c r="A62" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="B62" s="12" t="s">
+      <c r="B62" s="9" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A63" s="12" t="s">
+      <c r="A63" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="B63" s="12" t="s">
+      <c r="B63" s="9" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A64" s="12" t="s">
+      <c r="A64" s="9" t="s">
         <v>242</v>
       </c>
-      <c r="B64" s="12" t="s">
+      <c r="B64" s="9" t="s">
         <v>243</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A65" s="12" t="s">
+      <c r="A65" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="B65" s="12" t="s">
+      <c r="B65" s="9" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A66" s="12" t="s">
+      <c r="A66" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="B66" s="12" t="s">
+      <c r="B66" s="9" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A67" s="12" t="s">
+      <c r="A67" s="9" t="s">
         <v>240</v>
       </c>
-      <c r="B67" s="12" t="s">
+      <c r="B67" s="9" t="s">
         <v>241</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A68" s="12" t="s">
+      <c r="A68" s="9" t="s">
         <v>244</v>
       </c>
-      <c r="B68" s="12" t="s">
+      <c r="B68" s="9" t="s">
         <v>245</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A69" s="12" t="s">
+      <c r="A69" s="9" t="s">
         <v>114</v>
       </c>
-      <c r="B69" s="12" t="s">
+      <c r="B69" s="9" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A70" s="12" t="s">
+      <c r="A70" s="9" t="s">
         <v>116</v>
       </c>
-      <c r="B70" s="12" t="s">
+      <c r="B70" s="9" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A71" s="12" t="s">
+      <c r="A71" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="B71" s="12" t="s">
+      <c r="B71" s="9" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A72" s="12" t="s">
+      <c r="A72" s="9" t="s">
         <v>254</v>
       </c>
-      <c r="B72" s="12" t="s">
+      <c r="B72" s="9" t="s">
         <v>255</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A73" s="12" t="s">
+      <c r="A73" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="B73" s="12" t="s">
+      <c r="B73" s="9" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A74" s="12" t="s">
+      <c r="A74" s="9" t="s">
         <v>226</v>
       </c>
-      <c r="B74" s="12" t="s">
+      <c r="B74" s="9" t="s">
         <v>227</v>
       </c>
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A75" s="12" t="s">
+      <c r="A75" s="9" t="s">
         <v>120</v>
       </c>
-      <c r="B75" s="12" t="s">
+      <c r="B75" s="9" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A76" s="12" t="s">
+      <c r="A76" s="9" t="s">
         <v>122</v>
       </c>
-      <c r="B76" s="12" t="s">
+      <c r="B76" s="9" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A77" s="12" t="s">
+      <c r="A77" s="9" t="s">
         <v>124</v>
       </c>
-      <c r="B77" s="12" t="s">
+      <c r="B77" s="9" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A78" s="12" t="s">
+      <c r="A78" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="B78" s="12" t="s">
+      <c r="B78" s="9" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A79" s="12" t="s">
+      <c r="A79" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="B79" s="12" t="s">
+      <c r="B79" s="9" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A80" s="12" t="s">
+      <c r="A80" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="B80" s="12" t="s">
+      <c r="B80" s="9" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A81" s="12" t="s">
+      <c r="A81" s="9" t="s">
         <v>169</v>
       </c>
-      <c r="B81" s="12" t="s">
+      <c r="B81" s="9" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A82" s="12" t="s">
+      <c r="A82" s="9" t="s">
         <v>435</v>
       </c>
-      <c r="B82" s="12" t="s">
+      <c r="B82" s="9" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A83" s="12" t="s">
+      <c r="A83" s="9" t="s">
         <v>130</v>
       </c>
-      <c r="B83" s="12" t="s">
+      <c r="B83" s="9" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A84" s="12" t="s">
+      <c r="A84" s="9" t="s">
         <v>202</v>
       </c>
-      <c r="B84" s="12" t="s">
+      <c r="B84" s="9" t="s">
         <v>203</v>
       </c>
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A85" s="12" t="s">
+      <c r="A85" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="B85" s="12" t="s">
+      <c r="B85" s="9" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A86" s="12" t="s">
+      <c r="A86" s="9" t="s">
         <v>436</v>
       </c>
-      <c r="B86" s="12" t="s">
+      <c r="B86" s="9" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A87" s="12" t="s">
+      <c r="A87" s="9" t="s">
         <v>139</v>
       </c>
-      <c r="B87" s="12" t="s">
+      <c r="B87" s="9" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A88" s="12" t="s">
+      <c r="A88" s="9" t="s">
         <v>437</v>
       </c>
-      <c r="B88" s="12" t="s">
+      <c r="B88" s="9" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A89" s="12" t="s">
+      <c r="A89" s="9" t="s">
         <v>143</v>
       </c>
-      <c r="B89" s="12" t="s">
+      <c r="B89" s="9" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A90" s="12" t="s">
+      <c r="A90" s="9" t="s">
         <v>188</v>
       </c>
-      <c r="B90" s="12" t="s">
+      <c r="B90" s="9" t="s">
         <v>189</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A91" s="12" t="s">
+      <c r="A91" s="9" t="s">
         <v>134</v>
       </c>
-      <c r="B91" s="12" t="s">
+      <c r="B91" s="9" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A92" s="12" t="s">
+      <c r="A92" s="9" t="s">
         <v>204</v>
       </c>
-      <c r="B92" s="12" t="s">
+      <c r="B92" s="9" t="s">
         <v>205</v>
       </c>
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A93" s="12" t="s">
+      <c r="A93" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="B93" s="12" t="s">
+      <c r="B93" s="9" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A94" s="12" t="s">
+      <c r="A94" s="9" t="s">
         <v>220</v>
       </c>
-      <c r="B94" s="12" t="s">
+      <c r="B94" s="9" t="s">
         <v>221</v>
       </c>
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A95" s="12" t="s">
+      <c r="A95" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="B95" s="12" t="s">
+      <c r="B95" s="9" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A96" s="12" t="s">
+      <c r="A96" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="B96" s="12" t="s">
+      <c r="B96" s="9" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A97" s="12" t="s">
+      <c r="A97" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="B97" s="12" t="s">
+      <c r="B97" s="9" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="98" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A98" s="12" t="s">
+      <c r="A98" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="B98" s="12" t="s">
+      <c r="B98" s="9" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="99" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A99" s="12" t="s">
+      <c r="A99" s="9" t="s">
         <v>138</v>
       </c>
-      <c r="B99" s="12" t="s">
+      <c r="B99" s="9" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="100" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A100" s="12" t="s">
+      <c r="A100" s="9" t="s">
         <v>136</v>
       </c>
-      <c r="B100" s="12" t="s">
+      <c r="B100" s="9" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="101" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A101" s="12" t="s">
+      <c r="A101" s="9" t="s">
         <v>173</v>
       </c>
-      <c r="B101" s="12" t="s">
+      <c r="B101" s="9" t="s">
         <v>172</v>
       </c>
     </row>
     <row r="102" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A102" s="12" t="s">
+      <c r="A102" s="9" t="s">
         <v>171</v>
       </c>
-      <c r="B102" s="12" t="s">
+      <c r="B102" s="9" t="s">
         <v>172</v>
       </c>
     </row>
     <row r="103" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A103" s="12" t="s">
+      <c r="A103" s="9" t="s">
         <v>141</v>
       </c>
-      <c r="B103" s="12" t="s">
+      <c r="B103" s="9" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="104" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A104" s="12" t="s">
+      <c r="A104" s="9" t="s">
         <v>145</v>
       </c>
-      <c r="B104" s="12" t="s">
+      <c r="B104" s="9" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="105" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A105" s="12" t="s">
+      <c r="A105" s="9" t="s">
         <v>147</v>
       </c>
-      <c r="B105" s="12" t="s">
+      <c r="B105" s="9" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="106" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A106" s="12" t="s">
+      <c r="A106" s="9" t="s">
         <v>149</v>
       </c>
-      <c r="B106" s="12" t="s">
+      <c r="B106" s="9" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="107" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A107" s="12" t="s">
+      <c r="A107" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="B107" s="12" t="s">
+      <c r="B107" s="9" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="108" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A108" s="12" t="s">
+      <c r="A108" s="9" t="s">
         <v>100</v>
       </c>
-      <c r="B108" s="12" t="s">
+      <c r="B108" s="9" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="109" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A109" s="12" t="s">
+      <c r="A109" s="9" t="s">
         <v>102</v>
       </c>
-      <c r="B109" s="12" t="s">
+      <c r="B109" s="9" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="110" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A110" s="12" t="s">
+      <c r="A110" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="B110" s="12" t="s">
+      <c r="B110" s="9" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="111" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A111" s="12" t="s">
+      <c r="A111" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="B111" s="12" t="s">
+      <c r="B111" s="9" t="s">
         <v>152</v>
       </c>
     </row>
     <row r="112" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A112" s="12" t="s">
+      <c r="A112" s="9" t="s">
         <v>438</v>
       </c>
-      <c r="B112" s="12" t="s">
+      <c r="B112" s="9" t="s">
         <v>152</v>
       </c>
     </row>
     <row r="113" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A113" s="12" t="s">
+      <c r="A113" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="B113" s="12" t="s">
+      <c r="B113" s="9" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="114" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A114" s="12" t="s">
+      <c r="A114" s="9" t="s">
         <v>153</v>
       </c>
-      <c r="B114" s="12" t="s">
+      <c r="B114" s="9" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="115" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A115" s="12" t="s">
+      <c r="A115" s="9" t="s">
         <v>155</v>
       </c>
-      <c r="B115" s="12" t="s">
+      <c r="B115" s="9" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="116" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A116" s="12" t="s">
+      <c r="A116" s="9" t="s">
         <v>165</v>
       </c>
-      <c r="B116" s="12" t="s">
+      <c r="B116" s="9" t="s">
         <v>166</v>
       </c>
     </row>
     <row r="117" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A117" s="12" t="s">
+      <c r="A117" s="9" t="s">
         <v>167</v>
       </c>
-      <c r="B117" s="12" t="s">
+      <c r="B117" s="9" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="118" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A118" s="12" t="s">
+      <c r="A118" s="9" t="s">
         <v>218</v>
       </c>
-      <c r="B118" s="12" t="s">
+      <c r="B118" s="9" t="s">
         <v>219</v>
       </c>
     </row>
     <row r="119" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A119" s="12" t="s">
+      <c r="A119" s="9" t="s">
         <v>246</v>
       </c>
-      <c r="B119" s="12" t="s">
+      <c r="B119" s="9" t="s">
         <v>247</v>
       </c>
     </row>
     <row r="120" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A120" s="12" t="s">
+      <c r="A120" s="9" t="s">
         <v>174</v>
       </c>
-      <c r="B120" s="12" t="s">
+      <c r="B120" s="9" t="s">
         <v>175</v>
       </c>
     </row>
     <row r="121" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A121" s="12" t="s">
+      <c r="A121" s="9" t="s">
         <v>176</v>
       </c>
-      <c r="B121" s="12" t="s">
+      <c r="B121" s="9" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="122" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A122" s="12" t="s">
+      <c r="A122" s="9" t="s">
         <v>178</v>
       </c>
-      <c r="B122" s="12" t="s">
+      <c r="B122" s="9" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="123" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A123" s="12" t="s">
+      <c r="A123" s="9" t="s">
         <v>180</v>
       </c>
-      <c r="B123" s="12" t="s">
+      <c r="B123" s="9" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="124" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A124" s="12" t="s">
+      <c r="A124" s="9" t="s">
         <v>181</v>
       </c>
-      <c r="B124" s="12" t="s">
+      <c r="B124" s="9" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="125" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A125" s="12" t="s">
+      <c r="A125" s="9" t="s">
         <v>182</v>
       </c>
-      <c r="B125" s="12" t="s">
+      <c r="B125" s="9" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="126" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A126" s="12" t="s">
+      <c r="A126" s="9" t="s">
         <v>439</v>
       </c>
-      <c r="B126" s="12" t="s">
+      <c r="B126" s="9" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="127" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A127" s="12" t="s">
+      <c r="A127" s="9" t="s">
         <v>183</v>
       </c>
-      <c r="B127" s="12" t="s">
+      <c r="B127" s="9" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="128" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A128" s="12" t="s">
+      <c r="A128" s="9" t="s">
         <v>184</v>
       </c>
-      <c r="B128" s="12" t="s">
+      <c r="B128" s="9" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="129" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A129" s="12" t="s">
+      <c r="A129" s="9" t="s">
         <v>440</v>
       </c>
-      <c r="B129" s="12" t="s">
+      <c r="B129" s="9" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="130" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A130" s="12" t="s">
+      <c r="A130" s="9" t="s">
         <v>185</v>
       </c>
-      <c r="B130" s="12" t="s">
+      <c r="B130" s="9" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="131" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A131" s="12" t="s">
+      <c r="A131" s="9" t="s">
         <v>441</v>
       </c>
-      <c r="B131" s="12" t="s">
+      <c r="B131" s="9" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="132" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A132" s="12" t="s">
+      <c r="A132" s="9" t="s">
         <v>186</v>
       </c>
-      <c r="B132" s="12" t="s">
+      <c r="B132" s="9" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="133" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A133" s="12" t="s">
+      <c r="A133" s="9" t="s">
         <v>128</v>
       </c>
-      <c r="B133" s="12" t="s">
+      <c r="B133" s="9" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="134" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A134" s="12" t="s">
+      <c r="A134" s="9" t="s">
         <v>132</v>
       </c>
-      <c r="B134" s="12" t="s">
+      <c r="B134" s="9" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="135" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A135" s="12" t="s">
+      <c r="A135" s="9" t="s">
         <v>192</v>
       </c>
-      <c r="B135" s="12" t="s">
+      <c r="B135" s="9" t="s">
         <v>193</v>
       </c>
     </row>
     <row r="136" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A136" s="12" t="s">
+      <c r="A136" s="9" t="s">
         <v>194</v>
       </c>
-      <c r="B136" s="12" t="s">
+      <c r="B136" s="9" t="s">
         <v>195</v>
       </c>
     </row>
     <row r="137" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A137" s="12" t="s">
+      <c r="A137" s="9" t="s">
         <v>442</v>
       </c>
-      <c r="B137" s="12" t="s">
+      <c r="B137" s="9" t="s">
         <v>195</v>
       </c>
     </row>
     <row r="138" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A138" s="12" t="s">
+      <c r="A138" s="9" t="s">
         <v>190</v>
       </c>
-      <c r="B138" s="12" t="s">
+      <c r="B138" s="9" t="s">
         <v>191</v>
       </c>
     </row>
     <row r="139" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A139" s="12" t="s">
+      <c r="A139" s="9" t="s">
         <v>196</v>
       </c>
-      <c r="B139" s="12" t="s">
+      <c r="B139" s="9" t="s">
         <v>197</v>
       </c>
     </row>
     <row r="140" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A140" s="12" t="s">
+      <c r="A140" s="9" t="s">
         <v>206</v>
       </c>
-      <c r="B140" s="12" t="s">
+      <c r="B140" s="9" t="s">
         <v>207</v>
       </c>
     </row>
     <row r="141" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A141" s="12" t="s">
+      <c r="A141" s="9" t="s">
         <v>208</v>
       </c>
-      <c r="B141" s="12" t="s">
+      <c r="B141" s="9" t="s">
         <v>209</v>
       </c>
     </row>
     <row r="142" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A142" s="12" t="s">
+      <c r="A142" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="B142" s="12" t="s">
+      <c r="B142" s="9" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="143" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A143" s="12" t="s">
+      <c r="A143" s="9" t="s">
         <v>212</v>
       </c>
-      <c r="B143" s="12" t="s">
+      <c r="B143" s="9" t="s">
         <v>213</v>
       </c>
     </row>
     <row r="144" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A144" s="12" t="s">
+      <c r="A144" s="9" t="s">
         <v>214</v>
       </c>
-      <c r="B144" s="12" t="s">
+      <c r="B144" s="9" t="s">
         <v>215</v>
       </c>
     </row>
     <row r="145" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A145" s="12" t="s">
+      <c r="A145" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="B145" s="12" t="s">
+      <c r="B145" s="9" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="146" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A146" s="12" t="s">
+      <c r="A146" s="9" t="s">
         <v>159</v>
       </c>
-      <c r="B146" s="12" t="s">
+      <c r="B146" s="9" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="147" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A147" s="12" t="s">
+      <c r="A147" s="9" t="s">
         <v>161</v>
       </c>
-      <c r="B147" s="12" t="s">
+      <c r="B147" s="9" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="148" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A148" s="12" t="s">
+      <c r="A148" s="9" t="s">
         <v>163</v>
       </c>
-      <c r="B148" s="12" t="s">
+      <c r="B148" s="9" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="149" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A149" s="12" t="s">
+      <c r="A149" s="9" t="s">
         <v>228</v>
       </c>
-      <c r="B149" s="12" t="s">
+      <c r="B149" s="9" t="s">
         <v>228</v>
       </c>
     </row>
     <row r="150" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A150" s="12" t="s">
+      <c r="A150" s="9" t="s">
         <v>229</v>
       </c>
-      <c r="B150" s="12" t="s">
+      <c r="B150" s="9" t="s">
         <v>229</v>
       </c>
     </row>
     <row r="151" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A151" s="12" t="s">
+      <c r="A151" s="9" t="s">
         <v>216</v>
       </c>
-      <c r="B151" s="12" t="s">
+      <c r="B151" s="9" t="s">
         <v>217</v>
       </c>
     </row>
     <row r="152" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A152" s="12" t="s">
-        <v>500</v>
-      </c>
-      <c r="B152" s="12" t="s">
-        <v>501</v>
+      <c r="A152" s="9" t="s">
+        <v>491</v>
+      </c>
+      <c r="B152" s="9" t="s">
+        <v>492</v>
       </c>
     </row>
   </sheetData>
@@ -3906,50 +3997,50 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="10" t="s">
         <v>443</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="10" t="s">
         <v>444</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="9" t="s">
         <v>445</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="9" t="s">
         <v>199</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="9" t="s">
         <v>446</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="9" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="9" t="s">
         <v>447</v>
       </c>
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="9" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="9" t="s">
         <v>448</v>
       </c>
-      <c r="B5" s="12" t="s">
+      <c r="B5" s="9" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A6" s="12" t="s">
+      <c r="A6" s="9" t="s">
         <v>449</v>
       </c>
-      <c r="B6" s="12" t="s">
+      <c r="B6" s="9" t="s">
         <v>140</v>
       </c>
     </row>
@@ -3960,14 +4051,14 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47A3CEDA-FEC6-4ADF-A8A7-FE3D173EF629}">
-  <dimension ref="A1:B103"/>
+  <dimension ref="A1:B105"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="8" t="s">
         <v>1</v>
       </c>
     </row>
@@ -4572,7 +4663,7 @@
       </c>
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A77" s="9" t="s">
+      <c r="A77" s="7" t="s">
         <v>402</v>
       </c>
       <c r="B77" s="1" t="s">
@@ -4580,7 +4671,7 @@
       </c>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A78" s="9" t="s">
+      <c r="A78" s="7" t="s">
         <v>402</v>
       </c>
       <c r="B78" s="1" t="s">
@@ -4588,7 +4679,7 @@
       </c>
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A79" s="9" t="s">
+      <c r="A79" s="7" t="s">
         <v>402</v>
       </c>
       <c r="B79" s="1" t="s">
@@ -4596,7 +4687,7 @@
       </c>
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A80" s="9" t="s">
+      <c r="A80" s="7" t="s">
         <v>402</v>
       </c>
       <c r="B80" s="1" t="s">
@@ -4780,11 +4871,27 @@
       </c>
     </row>
     <row r="103" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A103" s="10" t="s">
+      <c r="A103" s="12" t="s">
         <v>489</v>
       </c>
       <c r="B103" s="1" t="s">
         <v>488</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A104" s="1" t="s">
+        <v>495</v>
+      </c>
+      <c r="B104" s="1" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A105" s="1" t="s">
+        <v>496</v>
+      </c>
+      <c r="B105" s="1" t="s">
+        <v>497</v>
       </c>
     </row>
   </sheetData>
@@ -4798,10 +4905,10 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="11" t="s">
         <v>443</v>
       </c>
-      <c r="B1" s="14" t="s">
+      <c r="B1" s="11" t="s">
         <v>444</v>
       </c>
     </row>
@@ -4875,108 +4982,44 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4AB1AC11-73D5-4AD4-B5BC-7F2393CC7475}">
-  <dimension ref="A1:D7"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{980D8F5D-6D83-45CB-A04A-C3A60B7CA15E}">
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="4" max="4" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
-        <v>464</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>465</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>466</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>467</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="13" t="s">
+        <v>509</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>511</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="15">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>468</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>469</v>
-      </c>
-      <c r="D2" s="2">
-        <v>1000000000</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="2">
-        <v>1</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>470</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>471</v>
-      </c>
-      <c r="D3" s="2">
-        <v>76000</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="2">
+      <c r="B2" s="15">
+        <v>0</v>
+      </c>
+      <c r="C2" s="15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="15">
         <v>2</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>468</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>472</v>
-      </c>
-      <c r="D4" s="2">
-        <v>500000000</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="2">
-        <v>2</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>470</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>473</v>
-      </c>
-      <c r="D5" s="2">
-        <v>38000</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="2">
-        <v>3</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>468</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>474</v>
-      </c>
-      <c r="D6" s="2">
-        <v>100000000</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="7">
-        <v>4</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>468</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>490</v>
-      </c>
-      <c r="D7" s="8">
+      <c r="B3" s="16">
+        <v>4000000000</v>
+      </c>
+      <c r="C3" s="16">
         <v>400000000</v>
       </c>
     </row>
@@ -4986,32 +5029,134 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32AEBD3E-E17A-4FD7-BDAF-3A1BA4999487}">
-  <dimension ref="A1:B3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6BF3446E-3AFE-40D0-805F-0CC526CADBC5}">
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="4.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.44140625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
-        <v>475</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>476</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
-        <v>477</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>425</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>478</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>426</v>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" s="14" t="s">
+        <v>464</v>
+      </c>
+      <c r="B1" s="14" t="s">
+        <v>465</v>
+      </c>
+      <c r="C1" s="14" t="s">
+        <v>466</v>
+      </c>
+      <c r="D1" s="14" t="s">
+        <v>467</v>
+      </c>
+      <c r="E1" s="14" t="s">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="17">
+        <v>1</v>
+      </c>
+      <c r="B2" s="17" t="s">
+        <v>468</v>
+      </c>
+      <c r="C2" s="17" t="s">
+        <v>469</v>
+      </c>
+      <c r="D2" s="18">
+        <v>1000000000</v>
+      </c>
+      <c r="E2" s="18" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="17">
+        <v>1</v>
+      </c>
+      <c r="B3" s="17" t="s">
+        <v>470</v>
+      </c>
+      <c r="C3" s="17" t="s">
+        <v>471</v>
+      </c>
+      <c r="D3" s="18">
+        <v>76000</v>
+      </c>
+      <c r="E3" s="18" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="17">
+        <v>2</v>
+      </c>
+      <c r="B4" s="17" t="s">
+        <v>468</v>
+      </c>
+      <c r="C4" s="17" t="s">
+        <v>472</v>
+      </c>
+      <c r="D4" s="18">
+        <v>500000000</v>
+      </c>
+      <c r="E4" s="18" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="17">
+        <v>2</v>
+      </c>
+      <c r="B5" s="17" t="s">
+        <v>470</v>
+      </c>
+      <c r="C5" s="17" t="s">
+        <v>473</v>
+      </c>
+      <c r="D5" s="18">
+        <v>38000</v>
+      </c>
+      <c r="E5" s="18" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="17">
+        <v>3</v>
+      </c>
+      <c r="B6" s="17" t="s">
+        <v>468</v>
+      </c>
+      <c r="C6" s="17" t="s">
+        <v>474</v>
+      </c>
+      <c r="D6" s="18">
+        <v>100000000</v>
+      </c>
+      <c r="E6" s="18" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" s="19">
+        <v>4</v>
+      </c>
+      <c r="B7" s="19" t="s">
+        <v>468</v>
+      </c>
+      <c r="C7" s="19" t="s">
+        <v>490</v>
+      </c>
+      <c r="D7" s="20">
+        <v>400000000</v>
+      </c>
+      <c r="E7" s="20" t="s">
+        <v>512</v>
       </c>
     </row>
   </sheetData>

</xml_diff>